<commit_message>
pruebas unitearias de backend + README
</commit_message>
<xml_diff>
--- a/samples/datos.xlsx
+++ b/samples/datos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdieg\OneDrive\Documentos\PersonalProjects\test_montefiori\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdieg\OneDrive\Documentos\PersonalProjects\test_montefiori\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F1EC6F1-FE96-484D-AB87-468FF66343E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501468A4-2160-43F8-89D8-6AAC71C84B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04220F85-8600-4111-8193-57C8AA91763E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>Nombre</t>
   </si>
@@ -96,6 +96,27 @@
   </si>
   <si>
     <t>M</t>
+  </si>
+  <si>
+    <t>Pepe@gmail.com</t>
+  </si>
+  <si>
+    <t>Juan@gmail.com</t>
+  </si>
+  <si>
+    <t>Ana@gmail.com</t>
+  </si>
+  <si>
+    <t>Ann@gmail.com</t>
+  </si>
+  <si>
+    <t>Marcelo@gmail.com</t>
+  </si>
+  <si>
+    <t>Kiara@gmail.com</t>
+  </si>
+  <si>
+    <t>Cesar@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -518,9 +539,8 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="str">
-        <f>A2&amp;"@gmail.com"</f>
-        <v>Pepe@gmail.com</v>
+      <c r="B2" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="C2" s="2">
         <v>999878797</v>
@@ -536,9 +556,8 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="str">
-        <f t="shared" ref="B3:B8" si="0">A3&amp;"@gmail.com"</f>
-        <v>Juan@gmail.com</v>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="C3" s="2">
         <v>959669874</v>
@@ -554,9 +573,8 @@
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Ana@gmail.com</v>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="C4" s="2">
         <v>999444120</v>
@@ -572,9 +590,8 @@
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Ann@gmail.com</v>
+      <c r="B5" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="C5" s="2">
         <v>998789877</v>
@@ -590,9 +607,8 @@
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Marcelo@gmail.com</v>
+      <c r="B6" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="C6" s="2">
         <v>963852741</v>
@@ -608,9 +624,8 @@
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Kiara@gmail.com</v>
+      <c r="B7" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="C7" s="2">
         <v>951478236</v>
@@ -626,9 +641,8 @@
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Cesar@gmail.com</v>
+      <c r="B8" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="C8" s="3">
         <v>987487588</v>

</xml_diff>